<commit_message>
chore: weekly deadline update
</commit_message>
<xml_diff>
--- a/data/Conferences.xlsx
+++ b/data/Conferences.xlsx
@@ -1565,57 +1565,57 @@
       <c r="K15" s="60" t="inlineStr"/>
     </row>
     <row r="16" ht="28.5" customHeight="1" s="37">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="38" t="inlineStr">
         <is>
           <t>安全</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="38" t="inlineStr">
         <is>
           <t>CCS</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="39" t="inlineStr">
         <is>
           <t>ACM Conference on Computer and Communications Security</t>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr">
+      <c r="D16" s="40" t="inlineStr">
         <is>
           <t>Atlanta，USA</t>
         </is>
       </c>
-      <c r="E16" s="15" t="inlineStr">
-        <is>
-          <t>October, TBD</t>
-        </is>
-      </c>
-      <c r="F16" s="14" t="inlineStr">
+      <c r="E16" s="41" t="inlineStr">
+        <is>
+          <t>10.11-10.15</t>
+        </is>
+      </c>
+      <c r="F16" s="40" t="inlineStr">
         <is>
           <t>北美</t>
         </is>
       </c>
-      <c r="G16" s="15" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H16" s="16" t="inlineStr">
+      <c r="G16" s="41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H16" s="42" t="inlineStr">
         <is>
           <t>ACM</t>
         </is>
       </c>
-      <c r="I16" s="17" t="inlineStr">
+      <c r="I16" s="43" t="inlineStr">
         <is>
           <t>https://dblp.org/db/conf/ccs/</t>
         </is>
       </c>
-      <c r="J16" s="67" t="inlineStr">
+      <c r="J16" s="44" t="inlineStr">
         <is>
           <t>https://www.sigsac.org/ccs/CCS2027/</t>
         </is>
       </c>
-      <c r="K16" s="69" t="inlineStr"/>
+      <c r="K16" s="58" t="inlineStr"/>
     </row>
     <row r="17" ht="42.75" customHeight="1" s="37">
       <c r="A17" s="13" t="inlineStr">
@@ -1671,57 +1671,57 @@
       <c r="K17" s="60" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="38" t="inlineStr">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>安全</t>
         </is>
       </c>
-      <c r="B18" s="38" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>S&amp;P</t>
         </is>
       </c>
-      <c r="C18" s="39" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>IEEE Symposium on Security and Privacy</t>
         </is>
       </c>
-      <c r="D18" s="40" t="inlineStr">
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>MONTREAL, CANADA</t>
         </is>
       </c>
-      <c r="E18" s="41" t="inlineStr">
+      <c r="E18" s="15" t="inlineStr">
         <is>
           <t>05.17-05.19</t>
         </is>
       </c>
-      <c r="F18" s="40" t="inlineStr">
+      <c r="F18" s="14" t="inlineStr">
         <is>
           <t>北美</t>
         </is>
       </c>
-      <c r="G18" s="40" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H18" s="42" t="inlineStr">
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H18" s="16" t="inlineStr">
         <is>
           <t>IEEE</t>
         </is>
       </c>
-      <c r="I18" s="43" t="inlineStr">
+      <c r="I18" s="17" t="inlineStr">
         <is>
           <t>https://dblp.org/db/conf/sp/</t>
         </is>
       </c>
-      <c r="J18" s="44" t="inlineStr">
+      <c r="J18" s="67" t="inlineStr">
         <is>
           <t>https://sp2027.ieee-security.org/index.html</t>
         </is>
       </c>
-      <c r="K18" s="58" t="inlineStr"/>
+      <c r="K18" s="69" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
@@ -2450,57 +2450,57 @@
       <c r="K32" s="60" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="38" t="inlineStr">
+      <c r="A33" s="13" t="inlineStr">
         <is>
           <t>数据库</t>
         </is>
       </c>
-      <c r="B33" s="38" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>SIGKDD</t>
         </is>
       </c>
-      <c r="C33" s="39" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>ACM SIGKDD Conference on Knowledge Discovery and Data Mining</t>
         </is>
       </c>
-      <c r="D33" s="40" t="inlineStr">
+      <c r="D33" s="14" t="inlineStr">
         <is>
           <t>San Jose, (California), USA</t>
         </is>
       </c>
-      <c r="E33" s="41" t="inlineStr">
+      <c r="E33" s="15" t="inlineStr">
         <is>
           <t>08.01-08.05</t>
         </is>
       </c>
-      <c r="F33" s="40" t="inlineStr">
+      <c r="F33" s="14" t="inlineStr">
         <is>
           <t>北美</t>
         </is>
       </c>
-      <c r="G33" s="40" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H33" s="42" t="inlineStr">
+      <c r="G33" s="14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H33" s="16" t="inlineStr">
         <is>
           <t>ACM</t>
         </is>
       </c>
-      <c r="I33" s="43" t="inlineStr">
+      <c r="I33" s="17" t="inlineStr">
         <is>
           <t>https://dblp.org/db/conf/kdd/</t>
         </is>
       </c>
-      <c r="J33" s="44" t="inlineStr">
+      <c r="J33" s="67" t="inlineStr">
         <is>
           <t>https://kdd2027.kdd.org/</t>
         </is>
       </c>
-      <c r="K33" s="56" t="inlineStr"/>
+      <c r="K33" s="60" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
@@ -2768,57 +2768,57 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="13" t="inlineStr">
+      <c r="A39" s="38" t="inlineStr">
         <is>
           <t>理论</t>
         </is>
       </c>
-      <c r="B39" s="13" t="inlineStr">
+      <c r="B39" s="38" t="inlineStr">
         <is>
           <t>CAV</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="C39" s="39" t="inlineStr">
         <is>
           <t>International Conference on Computer Aided Verification</t>
         </is>
       </c>
-      <c r="D39" s="14" t="inlineStr">
-        <is>
-          <t>Amsterdam, Netherlands</t>
-        </is>
-      </c>
-      <c r="E39" s="15" t="inlineStr">
-        <is>
-          <t>7.19-7.23</t>
-        </is>
-      </c>
-      <c r="F39" s="14" t="inlineStr">
+      <c r="D39" s="40" t="inlineStr">
+        <is>
+          <t>KIT, Amsterdam, The Netherlands</t>
+        </is>
+      </c>
+      <c r="E39" s="41" t="inlineStr">
+        <is>
+          <t>07.19-07.23</t>
+        </is>
+      </c>
+      <c r="F39" s="40" t="inlineStr">
         <is>
           <t>欧洲</t>
         </is>
       </c>
-      <c r="G39" s="14" t="inlineStr">
+      <c r="G39" s="40" t="inlineStr">
         <is>
           <t>2026.09.15</t>
         </is>
       </c>
-      <c r="H39" s="16" t="inlineStr">
+      <c r="H39" s="42" t="inlineStr">
         <is>
           <t>Springer</t>
         </is>
       </c>
-      <c r="I39" s="17" t="inlineStr">
+      <c r="I39" s="43" t="inlineStr">
         <is>
           <t>https://dblp.org/db/conf/cav/</t>
         </is>
       </c>
-      <c r="J39" s="67" t="inlineStr">
+      <c r="J39" s="44" t="inlineStr">
         <is>
           <t>https://conferences.i-cav.org/2027/</t>
         </is>
       </c>
-      <c r="K39" s="70" t="inlineStr">
+      <c r="K39" s="59" t="inlineStr">
         <is>
           <t>https://conferences.i-cav.org/2027/</t>
         </is>
@@ -2984,57 +2984,61 @@
       </c>
     </row>
     <row r="43" ht="28.5" customHeight="1" s="37">
-      <c r="A43" s="13" t="inlineStr">
+      <c r="A43" s="38" t="inlineStr">
         <is>
           <t>多媒体</t>
         </is>
       </c>
-      <c r="B43" s="13" t="inlineStr">
+      <c r="B43" s="38" t="inlineStr">
         <is>
           <t>IEEE VIS</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr">
+      <c r="C43" s="39" t="inlineStr">
         <is>
           <t>IEEE Visualization Conference</t>
         </is>
       </c>
-      <c r="D43" s="18" t="inlineStr">
+      <c r="D43" s="45" t="inlineStr">
         <is>
           <t>Chicago, USA</t>
         </is>
       </c>
-      <c r="E43" s="15" t="inlineStr">
+      <c r="E43" s="41" t="inlineStr">
         <is>
           <t>11.7-11.12</t>
         </is>
       </c>
-      <c r="F43" s="14" t="inlineStr">
+      <c r="F43" s="40" t="inlineStr">
         <is>
           <t>北美</t>
         </is>
       </c>
-      <c r="G43" s="14" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H43" s="16" t="inlineStr">
+      <c r="G43" s="40" t="inlineStr">
+        <is>
+          <t>2026.06.25</t>
+        </is>
+      </c>
+      <c r="H43" s="42" t="inlineStr">
         <is>
           <t>IEEE</t>
         </is>
       </c>
-      <c r="I43" s="17" t="inlineStr">
+      <c r="I43" s="43" t="inlineStr">
         <is>
           <t>https://dblp.org/db/conf/visualization/</t>
         </is>
       </c>
-      <c r="J43" s="6" t="inlineStr">
+      <c r="J43" s="46" t="inlineStr">
         <is>
           <t>https://www.computer.org/communities/vgtc</t>
         </is>
       </c>
-      <c r="K43" s="60" t="inlineStr"/>
+      <c r="K43" s="59" t="inlineStr">
+        <is>
+          <t>https://vis4climate.ivia.ch/workshop</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
@@ -3090,57 +3094,57 @@
       <c r="K44" s="60" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="38" t="inlineStr">
+      <c r="A45" s="13" t="inlineStr">
         <is>
           <t>软工</t>
         </is>
       </c>
-      <c r="B45" s="38" t="inlineStr">
+      <c r="B45" s="13" t="inlineStr">
         <is>
           <t>ISSTA</t>
         </is>
       </c>
-      <c r="C45" s="39" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr">
         <is>
           <t>International Symposium on Software Testing and Analysis</t>
         </is>
       </c>
-      <c r="D45" s="40" t="inlineStr">
+      <c r="D45" s="14" t="inlineStr">
         <is>
           <t>Singapore</t>
         </is>
       </c>
-      <c r="E45" s="41" t="inlineStr">
+      <c r="E45" s="15" t="inlineStr">
         <is>
           <t>09.07-09.10</t>
         </is>
       </c>
-      <c r="F45" s="40" t="inlineStr">
+      <c r="F45" s="14" t="inlineStr">
         <is>
           <t>亚太</t>
         </is>
       </c>
-      <c r="G45" s="40" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H45" s="42" t="inlineStr">
+      <c r="G45" s="14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H45" s="16" t="inlineStr">
         <is>
           <t>ACM</t>
         </is>
       </c>
-      <c r="I45" s="43" t="inlineStr">
+      <c r="I45" s="17" t="inlineStr">
         <is>
           <t>https://dblp.org/db/conf/issta/</t>
         </is>
       </c>
-      <c r="J45" s="44" t="inlineStr">
+      <c r="J45" s="67" t="inlineStr">
         <is>
           <t>https://conf.researchr.org/home/issta-2027</t>
         </is>
       </c>
-      <c r="K45" s="56" t="inlineStr"/>
+      <c r="K45" s="60" t="inlineStr"/>
     </row>
     <row r="46" ht="27" customHeight="1" s="37">
       <c r="A46" s="13" t="inlineStr">
@@ -3302,57 +3306,57 @@
       <c r="K48" s="60" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="13" t="inlineStr">
+      <c r="A49" s="38" t="inlineStr">
         <is>
           <t>AI</t>
         </is>
       </c>
-      <c r="B49" s="13" t="inlineStr">
+      <c r="B49" s="38" t="inlineStr">
         <is>
           <t>CVPR</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr">
+      <c r="C49" s="39" t="inlineStr">
         <is>
           <t>IEEE/CVF Computer Vision and Pattern Recognition Conference</t>
         </is>
       </c>
-      <c r="D49" s="14" t="inlineStr">
-        <is>
-          <t>Seattle, USA</t>
-        </is>
-      </c>
-      <c r="E49" s="15" t="inlineStr">
-        <is>
-          <t>6.20-6.24</t>
-        </is>
-      </c>
-      <c r="F49" s="14" t="inlineStr">
+      <c r="D49" s="40" t="inlineStr">
+        <is>
+          <t>Seattle, WA, United States</t>
+        </is>
+      </c>
+      <c r="E49" s="41" t="inlineStr">
+        <is>
+          <t>06.20-06.24</t>
+        </is>
+      </c>
+      <c r="F49" s="40" t="inlineStr">
         <is>
           <t>北美</t>
         </is>
       </c>
-      <c r="G49" s="14" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H49" s="16" t="inlineStr">
+      <c r="G49" s="40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H49" s="42" t="inlineStr">
         <is>
           <t>IEEE</t>
         </is>
       </c>
-      <c r="I49" s="17" t="inlineStr">
+      <c r="I49" s="43" t="inlineStr">
         <is>
           <t>https://dblp.org/db/conf/cvpr/</t>
         </is>
       </c>
-      <c r="J49" s="6" t="inlineStr">
-        <is>
-          <t>https://www.thecvf.com/?p=137</t>
-        </is>
-      </c>
-      <c r="K49" s="60" t="inlineStr"/>
+      <c r="J49" s="44" t="inlineStr">
+        <is>
+          <t>https://cvpr.thecvf.com/Conferences/2027</t>
+        </is>
+      </c>
+      <c r="K49" s="56" t="inlineStr"/>
     </row>
     <row r="50" ht="28.5" customHeight="1" s="37">
       <c r="A50" s="13" t="inlineStr">
@@ -3761,7 +3765,7 @@
       </c>
       <c r="J57" s="44" t="inlineStr">
         <is>
-          <t>https://acmweb2027.org/</t>
+          <t>https://www2027.thewebconf.org/</t>
         </is>
       </c>
       <c r="K57" s="59" t="inlineStr">
@@ -4086,111 +4090,111 @@
       <c r="K63" s="65" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="52" t="inlineStr">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>系统</t>
         </is>
       </c>
-      <c r="B64" s="52" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>MLsys</t>
         </is>
       </c>
-      <c r="C64" s="39" t="inlineStr">
+      <c r="C64" s="3" t="inlineStr">
         <is>
           <t>Conference on Machine Learning and Systems</t>
         </is>
       </c>
-      <c r="D64" s="53" t="inlineStr">
+      <c r="D64" s="4" t="inlineStr">
         <is>
           <t>Bellevue, (Washington), USA</t>
         </is>
       </c>
-      <c r="E64" s="53" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F64" s="53" t="inlineStr">
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
         <is>
           <t>北美</t>
         </is>
       </c>
-      <c r="G64" s="73" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H64" s="39" t="inlineStr">
+      <c r="G64" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
         <is>
           <t>MLSys/PMLR</t>
         </is>
       </c>
-      <c r="I64" s="46" t="inlineStr">
+      <c r="I64" s="6" t="inlineStr">
         <is>
           <t>https://mlsys.org/</t>
         </is>
       </c>
-      <c r="J64" s="44" t="inlineStr">
+      <c r="J64" s="67" t="inlineStr">
         <is>
           <t>https://mlsys.org/</t>
         </is>
       </c>
-      <c r="K64" s="63" t="inlineStr"/>
+      <c r="K64" s="65" t="inlineStr"/>
     </row>
     <row r="65" ht="29" customHeight="1" s="37">
-      <c r="A65" s="52" t="inlineStr">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>网络</t>
         </is>
       </c>
-      <c r="B65" s="52" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>MobiSys</t>
         </is>
       </c>
-      <c r="C65" s="39" t="inlineStr">
+      <c r="C65" s="3" t="inlineStr">
         <is>
           <t>ACM International Conference on Mobile Systems,
 Applications, and Services</t>
         </is>
       </c>
-      <c r="D65" s="53" t="inlineStr">
+      <c r="D65" s="4" t="inlineStr">
         <is>
           <t>Ho Chi Minh City, Vietnam Important Dates TPC Self Nomination TBA Abstract Registration TBA Paper Submission TBA Early Rejection Notification TBA Rebuttal Period TBA Final Decision Notification TBA Final Camera-ready Deadline TBA IoT Day TBA Rising Stars Forum TBA N</t>
         </is>
       </c>
-      <c r="E65" s="53" t="inlineStr">
+      <c r="E65" s="4" t="inlineStr">
         <is>
           <t>06.21-06.25</t>
         </is>
       </c>
-      <c r="F65" s="53" t="inlineStr">
+      <c r="F65" s="4" t="inlineStr">
         <is>
           <t>亚太</t>
         </is>
       </c>
-      <c r="G65" s="73" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H65" s="39" t="inlineStr">
+      <c r="G65" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
         <is>
           <t>ACM</t>
         </is>
       </c>
-      <c r="I65" s="46" t="inlineStr">
+      <c r="I65" s="6" t="inlineStr">
         <is>
           <t>http://dblp.uni-trier.de/db/conf/mobisys/</t>
         </is>
       </c>
-      <c r="J65" s="44" t="inlineStr">
+      <c r="J65" s="67" t="inlineStr">
         <is>
           <t>https://www.sigmobile.org/mobisys/2027/</t>
         </is>
       </c>
-      <c r="K65" s="63" t="inlineStr"/>
+      <c r="K65" s="65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -5729,77 +5733,78 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K57" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I62" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J65" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I66" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K78" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I79" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J82" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I84" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I85" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J85" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I86" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K57" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I62" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J65" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I66" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K78" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I79" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J82" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I84" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I85" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J85" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I86" r:id="rId150"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.7480314960629921" right="0.7480314960629921" top="0.984251968503937" bottom="0.984251968503937" header="0.5118110236220472" footer="0.5118110236220472"/>
@@ -5821,7 +5826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E151"/>
+  <dimension ref="A1:E152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9570,29 +9575,56 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" t="inlineStr">
+      <c r="A151" s="0" t="inlineStr">
         <is>
           <t>WWW</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr">
+      <c r="B151" s="0" t="inlineStr">
         <is>
           <t>Workshop Submission Deadline（2027）</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr">
+      <c r="C151" s="0" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D151" s="0" t="inlineStr">
         <is>
           <t>2027.02.16</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr">
+      <c r="E151" s="0" t="inlineStr">
         <is>
           <t>2026-08-31 12:01 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>IEEE VIS</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Workshop Submission Deadline（2027）</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>2026.06.25</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>2026-09-07 10:55 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>